<commit_message>
Merge spin tables and refine dev cheats
</commit_message>
<xml_diff>
--- a/ExcelTable/Cheat.xlsx
+++ b/ExcelTable/Cheat.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CheatCommands" sheetId="1" r:id="Rfa0f823a18424209"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CheatCommands" sheetId="1" r:id="Rab92d637851f43a9"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -352,15 +352,14 @@
   <x:cols>
     <x:col min="1" max="1" width="21.25" hidden="0" customWidth="1"/>
     <x:col min="2" max="2" width="16.25" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="23.75" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="45" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="26.25" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="23.75" hidden="0" customWidth="1"/>
-    <x:col min="7" max="7" width="16.25" hidden="0" customWidth="1"/>
-    <x:col min="8" max="8" width="13.75" hidden="0" customWidth="1"/>
-    <x:col min="9" max="9" width="23.75" hidden="0" customWidth="1"/>
-    <x:col min="10" max="10" width="12.5" hidden="0" customWidth="1"/>
-    <x:col min="11" max="11" width="45" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="35" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="26.25" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="23.75" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="16.25" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="13.75" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="23.75" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="12.5" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="45" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1">
@@ -371,30 +370,27 @@
         <x:v>CheatCode</x:v>
       </x:c>
       <x:c r="C1" s="12" t="str">
-        <x:v>DisplayName</x:v>
+        <x:v>Description</x:v>
       </x:c>
       <x:c r="D1" s="12" t="str">
-        <x:v>Description</x:v>
+        <x:v>CheatType</x:v>
       </x:c>
       <x:c r="E1" s="12" t="str">
-        <x:v>CheatType</x:v>
+        <x:v>TargetKey</x:v>
       </x:c>
       <x:c r="F1" s="12" t="str">
-        <x:v>TargetKey</x:v>
+        <x:v>ForceResultKey</x:v>
       </x:c>
       <x:c r="G1" s="12" t="str">
-        <x:v>ForceResultKey</x:v>
+        <x:v>UseCount</x:v>
       </x:c>
       <x:c r="H1" s="12" t="str">
-        <x:v>UseCount</x:v>
+        <x:v>RequiredRuntimeKind</x:v>
       </x:c>
       <x:c r="I1" s="12" t="str">
-        <x:v>RequiredRuntimeKind</x:v>
+        <x:v>Enabled</x:v>
       </x:c>
       <x:c r="J1" s="12" t="str">
-        <x:v>Enabled</x:v>
-      </x:c>
-      <x:c r="K1" s="12" t="str">
         <x:v>Notes</x:v>
       </x:c>
     </x:row>
@@ -427,9 +423,6 @@
         <x:v>client</x:v>
       </x:c>
       <x:c r="J2" s="13" t="str">
-        <x:v>client</x:v>
-      </x:c>
-      <x:c r="K2" s="13" t="str">
         <x:v>design</x:v>
       </x:c>
     </x:row>
@@ -441,30 +434,27 @@
         <x:v>테스트 UI 입력창에 입력할 치트 코드입니다.</x:v>
       </x:c>
       <x:c r="C3" s="14" t="str">
-        <x:v>테스트 UI 목록에 표시할 치트 이름입니다.</x:v>
+        <x:v>치트의 동작을 설명하는 목록 표시 문구입니다.</x:v>
       </x:c>
       <x:c r="D3" s="14" t="str">
-        <x:v>치트의 동작을 설명하는 목록 표시 문구입니다.</x:v>
+        <x:v>런타임에서 처리할 치트 동작 타입입니다.</x:v>
       </x:c>
       <x:c r="E3" s="14" t="str">
-        <x:v>런타임에서 처리할 치트 동작 타입입니다.</x:v>
+        <x:v>치트가 대상으로 삼는 슬롯 기능 또는 트리거 키입니다.</x:v>
       </x:c>
       <x:c r="F3" s="14" t="str">
-        <x:v>치트가 대상으로 삼는 슬롯 기능 또는 트리거 키입니다.</x:v>
+        <x:v>강제 결과가 필요한 치트에서 사용할 결과 키입니다.</x:v>
       </x:c>
       <x:c r="G3" s="14" t="str">
-        <x:v>강제 결과가 필요한 치트에서 사용할 결과 키입니다.</x:v>
+        <x:v>치트 입력 1회로 현재 플레이 세션에 부여할 사용 가능 횟수입니다.</x:v>
       </x:c>
       <x:c r="H3" s="14" t="str">
-        <x:v>치트 입력 1회로 현재 플레이 세션에 부여할 사용 가능 횟수입니다.</x:v>
+        <x:v>치트가 허용되는 런타임 종류입니다.</x:v>
       </x:c>
       <x:c r="I3" s="14" t="str">
-        <x:v>치트가 허용되는 런타임 종류입니다.</x:v>
+        <x:v>현재 치트 행을 사용할지 여부입니다.</x:v>
       </x:c>
       <x:c r="J3" s="14" t="str">
-        <x:v>현재 치트 행을 사용할지 여부입니다.</x:v>
-      </x:c>
-      <x:c r="K3" s="14" t="str">
         <x:v>개발 로직에서는 사용하지 않는 기획 참고 메모입니다.</x:v>
       </x:c>
     </x:row>
@@ -488,18 +478,15 @@
         <x:v>string</x:v>
       </x:c>
       <x:c r="G4" s="15" t="str">
-        <x:v>string</x:v>
+        <x:v>int</x:v>
       </x:c>
       <x:c r="H4" s="15" t="str">
-        <x:v>int</x:v>
+        <x:v>string</x:v>
       </x:c>
       <x:c r="I4" s="15" t="str">
-        <x:v>string</x:v>
+        <x:v>bool</x:v>
       </x:c>
       <x:c r="J4" s="15" t="str">
-        <x:v>bool</x:v>
-      </x:c>
-      <x:c r="K4" s="15" t="str">
         <x:v>string</x:v>
       </x:c>
     </x:row>
@@ -511,30 +498,27 @@
         <x:v>777</x:v>
       </x:c>
       <x:c r="C5" s="16" t="str">
-        <x:v>Force 777 Bonus</x:v>
+        <x:v>Force Wild x5 bonus entry and first 777 result once.</x:v>
       </x:c>
       <x:c r="D5" s="16" t="str">
-        <x:v>Force Wild x5 bonus entry and first 777 result once.</x:v>
+        <x:v>FORCE_777_BONUS_ONCE</x:v>
       </x:c>
       <x:c r="E5" s="16" t="str">
-        <x:v>FORCE_777_BONUS_ONCE</x:v>
+        <x:v>WILD_5_BONUS_SLOT</x:v>
       </x:c>
       <x:c r="F5" s="16" t="str">
-        <x:v>WILD_5_BONUS_SLOT</x:v>
-      </x:c>
-      <x:c r="G5" s="16" t="str">
         <x:v>777</x:v>
       </x:c>
-      <x:c r="H5" s="16" t="n">
+      <x:c r="G5" s="16" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="I5" s="16" t="str">
+      <x:c r="H5" s="16" t="str">
         <x:v>TEST_SANDBOX</x:v>
       </x:c>
-      <x:c r="J5" s="17" t="b">
+      <x:c r="I5" s="17" t="b">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="K5" s="16" t="str">
+      <x:c r="J5" s="16" t="str">
         <x:v>Development-only session cheat; release runtime cannot apply it.</x:v>
       </x:c>
     </x:row>

</xml_diff>